<commit_message>
Guardar en 1_PRESSUPOSTOS por código de cliente y PDF cliente junto al presupuesto
- La carpeta elegida contiene 0_PROGRAMA (app y catálogo) y 1_PRESSUPOSTOS
- Campo «Código cliente»: se guarda en 1_PRESSUPOSTOS/<código>/; sin código
  o 1000, en 1000/<Nombre - Teléfono>/. Se crean las carpetas que falten
- .json y .pdf con el mismo nombre (AAAA-NNN - Cliente); si cambia el código
  o el nombre, ambos se mueven
- PDF cliente generado como archivo (html2canvas + jsPDF, incluidos en lib/)
  y guardado automáticamente, con cortes de página entre filas
- Numeración y Abrir recorren todas las carpetas de clientes

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MHBE3gE6AFc5rMzkXkJrid
</commit_message>
<xml_diff>
--- a/plantilla_presupuesto.xlsx
+++ b/plantilla_presupuesto.xlsx
@@ -500,7 +500,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -516,7 +516,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Cliente</v>
+        <v>Código cliente (vacío o 1000 = sin código)</v>
       </c>
       <c r="B2" t="str">
         <v/>
@@ -524,7 +524,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Contacto</v>
+        <v>Cliente</v>
       </c>
       <c r="B3" t="str">
         <v/>
@@ -532,7 +532,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Referencia</v>
+        <v>Contacto</v>
       </c>
       <c r="B4" t="str">
         <v/>
@@ -540,7 +540,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Descripción</v>
+        <v>Referencia</v>
       </c>
       <c r="B5" t="str">
         <v/>
@@ -548,15 +548,23 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>Descripción</v>
+      </c>
+      <c r="B6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
         <v>Descuento carpintero (Sí / No)</v>
       </c>
-      <c r="B6" t="str">
+      <c r="B7" t="str">
         <v>No</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>